<commit_message>
Site rebuild from the City (CORE action) 2026-10-29 19:16
</commit_message>
<xml_diff>
--- a/free/small-business-invoice-template.xlsx
+++ b/free/small-business-invoice-template.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Use" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ready-made for your trade" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="ServiceList">Services!$B$6:$B$40</definedName>
@@ -30,7 +31,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.##"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -148,6 +149,21 @@
       <color rgb="00222831"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <color rgb="001F6FEB"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -182,7 +198,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -219,11 +235,27 @@
         <color rgb="00D9DEE7"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9DEE7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9DEE7"/>
+      </top>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -387,6 +419,20 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -881,6 +927,9 @@
           <t>[Job site or project name]</t>
         </is>
       </c>
+      <c r="E12" s="58" t="n"/>
+      <c r="F12" s="58" t="n"/>
+      <c r="G12" s="58" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="14" t="inlineStr">
@@ -893,6 +942,9 @@
           <t>[Street Address]</t>
         </is>
       </c>
+      <c r="E13" s="58" t="n"/>
+      <c r="F13" s="58" t="n"/>
+      <c r="G13" s="58" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="14" t="inlineStr">
@@ -905,6 +957,9 @@
           <t>[City, State ZIP]</t>
         </is>
       </c>
+      <c r="E14" s="58" t="n"/>
+      <c r="F14" s="58" t="n"/>
+      <c r="G14" s="58" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="14" t="inlineStr">
@@ -1293,12 +1348,12 @@
       </c>
     </row>
     <row r="38" ht="19" customHeight="1">
-      <c r="E38" s="34" t="inlineStr">
+      <c r="E38" s="65" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="F38" s="35" t="n"/>
+      <c r="F38" s="59" t="n"/>
       <c r="G38" s="36">
         <f>G35-G36+G37</f>
         <v/>
@@ -1320,7 +1375,6 @@
           <t>BALANCE DUE</t>
         </is>
       </c>
-      <c r="F40" s="1" t="n"/>
       <c r="G40" s="38">
         <f>G38-G39</f>
         <v/>
@@ -1354,8 +1408,8 @@
     <mergeCell ref="E35:F35"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="E38:F38"/>
+    <mergeCell ref="D12:G12"/>
     <mergeCell ref="E7:F7"/>
-    <mergeCell ref="D12:G12"/>
     <mergeCell ref="B44:G44"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="E37:F37"/>
@@ -1515,6 +1569,9 @@
           <t>[Job site or project name]</t>
         </is>
       </c>
+      <c r="E12" s="58" t="n"/>
+      <c r="F12" s="58" t="n"/>
+      <c r="G12" s="58" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="14" t="inlineStr">
@@ -1527,6 +1584,9 @@
           <t>[Street Address]</t>
         </is>
       </c>
+      <c r="E13" s="58" t="n"/>
+      <c r="F13" s="58" t="n"/>
+      <c r="G13" s="58" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="14" t="inlineStr">
@@ -1539,6 +1599,9 @@
           <t>[City, State ZIP]</t>
         </is>
       </c>
+      <c r="E14" s="58" t="n"/>
+      <c r="F14" s="58" t="n"/>
+      <c r="G14" s="58" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="14" t="inlineStr">
@@ -1927,12 +1990,12 @@
       </c>
     </row>
     <row r="38" ht="19" customHeight="1">
-      <c r="E38" s="34" t="inlineStr">
+      <c r="E38" s="65" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="F38" s="35" t="n"/>
+      <c r="F38" s="59" t="n"/>
       <c r="G38" s="36">
         <f>G35-G36+G37</f>
         <v/>
@@ -1944,7 +2007,6 @@
           <t>ESTIMATE TOTAL</t>
         </is>
       </c>
-      <c r="F39" s="1" t="n"/>
       <c r="G39" s="38">
         <f>G38</f>
         <v/>
@@ -2617,4 +2679,193 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="60" t="inlineStr">
+        <is>
+          <t>Want this ready-made for your trade?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>Each kit comes with your trade's services already filled in, an estimate tab and fillable PDFs; most also include 8 matching social media posts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="62" t="inlineStr">
+        <is>
+          <t>Business kit</t>
+        </is>
+      </c>
+      <c r="B4" s="62" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Car Detailing Business Kit</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>$9.99</t>
+        </is>
+      </c>
+      <c r="C5" s="63" t="inlineStr">
+        <is>
+          <t>https://the-fixer.org/p/car-detailing-business-kit/?from=free-xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DJ Booking Kit</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>$9.99</t>
+        </is>
+      </c>
+      <c r="C6" s="63" t="inlineStr">
+        <is>
+          <t>https://the-fixer.org/p/dj-booking-kit/?from=free-xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Dog Walking Business Kit</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>$9.99</t>
+        </is>
+      </c>
+      <c r="C7" s="63" t="inlineStr">
+        <is>
+          <t>https://the-fixer.org/p/dog-walking-business-kit/?from=free-xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>House Cleaning Business Kit</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>$9.99</t>
+        </is>
+      </c>
+      <c r="C8" s="63" t="inlineStr">
+        <is>
+          <t>https://the-fixer.org/p/house-cleaning-business-kit/?from=free-xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Personal Trainer Business Kit</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>$9.99</t>
+        </is>
+      </c>
+      <c r="C9" s="63" t="inlineStr">
+        <is>
+          <t>https://the-fixer.org/p/personal-trainer-business-kit/?from=free-xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Pet Grooming Business Kit</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>$9.99</t>
+        </is>
+      </c>
+      <c r="C10" s="63" t="inlineStr">
+        <is>
+          <t>https://the-fixer.org/p/pet-grooming-business-kit/?from=free-xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Plumbing Business Kit</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>$9.99</t>
+        </is>
+      </c>
+      <c r="C11" s="63" t="inlineStr">
+        <is>
+          <t>https://the-fixer.org/p/plumbing-business-kit/?from=free-xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="64" t="inlineStr">
+        <is>
+          <t>Every template: https://the-fixer.org</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>